<commit_message>
new spatial lag features and combined notebook 5 and 6
</commit_message>
<xml_diff>
--- a/dataset information/All variables and missing percentage.xlsx
+++ b/dataset information/All variables and missing percentage.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aukehilbrands/Documents/Studie/Thesis/dataset information/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0910A03-4819-EC42-AE17-DA44047449C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAFB6432-D19A-C443-935F-3034434BD050}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="820" windowWidth="28040" windowHeight="17440" xr2:uid="{B1AAE110-6AF2-834C-9804-2F2ED44668A0}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="149">
   <si>
     <t>Variabelenaam</t>
   </si>
@@ -443,24 +443,9 @@
     <t>pst_mvp: Meest voorkomende postcode</t>
   </si>
   <si>
-    <t>bev_dich</t>
-  </si>
-  <si>
-    <t>g_wozbag</t>
-  </si>
-  <si>
-    <t>p_huurw</t>
-  </si>
-  <si>
-    <t>a_soz_wb</t>
-  </si>
-  <si>
     <t>a_bedv</t>
   </si>
   <si>
-    <t>ste_oad</t>
-  </si>
-  <si>
     <t>Selection for spatial features</t>
   </si>
   <si>
@@ -480,6 +465,24 @@
   </si>
   <si>
     <t>a_ons_hbo: Studenten hbo</t>
+  </si>
+  <si>
+    <t>a_inw</t>
+  </si>
+  <si>
+    <t>a_woning</t>
+  </si>
+  <si>
+    <t>a_pau</t>
+  </si>
+  <si>
+    <t>a_opp_ha</t>
+  </si>
+  <si>
+    <t>a_ll</t>
+  </si>
+  <si>
+    <t>a_ll: Totaal leerlingen en studenten</t>
   </si>
 </sst>
 </file>
@@ -578,7 +581,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -592,6 +595,7 @@
     <xf numFmtId="10" fontId="8" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="10" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -927,15 +931,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7CAD586-3C0E-A245-A536-319D6F2F5747}">
-  <dimension ref="A1:F140"/>
+  <dimension ref="A1:G140"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="76.83203125" customWidth="1"/>
     <col min="2" max="2" width="4.5" customWidth="1"/>
     <col min="3" max="3" width="18.5" style="9" customWidth="1"/>
+    <col min="5" max="5" width="18.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -944,29 +949,35 @@
         <v>130</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+        <v>130</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="9">
+        <v>0</v>
+      </c>
+      <c r="E2" s="13">
+        <v>0</v>
+      </c>
+      <c r="F2" t="s">
         <v>143</v>
       </c>
-      <c r="B2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" s="9">
-        <v>0</v>
-      </c>
-      <c r="E2" t="s">
-        <v>135</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G2" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>2</v>
@@ -974,9 +985,17 @@
       <c r="C3" s="9">
         <v>0</v>
       </c>
-      <c r="F3" s="1"/>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E3" s="13">
+        <v>0</v>
+      </c>
+      <c r="F3" t="s">
+        <v>144</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>1</v>
       </c>
@@ -986,14 +1005,17 @@
       <c r="C4" s="9">
         <v>0</v>
       </c>
-      <c r="E4" t="s">
-        <v>136</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E4" s="13">
+        <v>0</v>
+      </c>
+      <c r="F4" t="s">
+        <v>147</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -1003,14 +1025,17 @@
       <c r="C5" s="9">
         <v>0</v>
       </c>
-      <c r="E5" t="s">
-        <v>137</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E5" s="13">
+        <v>0</v>
+      </c>
+      <c r="F5" t="s">
+        <v>135</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
@@ -1020,9 +1045,17 @@
       <c r="C6" s="9">
         <v>0</v>
       </c>
-      <c r="F6" s="1"/>
-    </row>
-    <row r="7" spans="1:6" s="6" customFormat="1" ht="22" x14ac:dyDescent="0.3">
+      <c r="E6" s="13">
+        <v>0</v>
+      </c>
+      <c r="F6" t="s">
+        <v>145</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" s="6" customFormat="1" ht="22" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
         <v>5</v>
       </c>
@@ -1030,14 +1063,17 @@
         <f>AVERAGE(C8:C37)</f>
         <v>2.6633333333333331E-3</v>
       </c>
-      <c r="E7" t="s">
-        <v>138</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E7" s="13">
+        <v>0</v>
+      </c>
+      <c r="F7" t="s">
+        <v>146</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>6</v>
       </c>
@@ -1048,7 +1084,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
@@ -1058,14 +1094,10 @@
       <c r="C9" s="9">
         <v>0</v>
       </c>
-      <c r="E9" t="s">
-        <v>139</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E9" s="9"/>
+      <c r="G9" s="1"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
@@ -1075,9 +1107,9 @@
       <c r="C10" s="9">
         <v>0</v>
       </c>
-      <c r="F10" s="1"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G10" s="1"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>9</v>
       </c>
@@ -1087,14 +1119,10 @@
       <c r="C11" s="9">
         <v>0</v>
       </c>
-      <c r="E11" t="s">
-        <v>140</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E11" s="9"/>
+      <c r="G11" s="3"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>10</v>
       </c>
@@ -1105,7 +1133,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>11</v>
       </c>
@@ -1116,7 +1144,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>12</v>
       </c>
@@ -1127,7 +1155,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>13</v>
       </c>
@@ -1138,7 +1166,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>14</v>
       </c>
@@ -1149,7 +1177,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>15</v>
       </c>
@@ -1160,7 +1188,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
         <v>16</v>
       </c>
@@ -1170,9 +1198,8 @@
       <c r="C18" s="9">
         <v>0</v>
       </c>
-      <c r="F18" s="3"/>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>17</v>
       </c>
@@ -1183,7 +1210,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
         <v>18</v>
       </c>
@@ -1194,7 +1221,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
         <v>19</v>
       </c>
@@ -1205,7 +1232,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
         <v>20</v>
       </c>
@@ -1215,8 +1242,9 @@
       <c r="C22" s="9">
         <v>0</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E22" s="13"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
         <v>21</v>
       </c>
@@ -1226,9 +1254,10 @@
       <c r="C23" s="9">
         <v>0</v>
       </c>
-      <c r="F23" s="3"/>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E23" s="13"/>
+      <c r="G23" s="3"/>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
         <v>22</v>
       </c>
@@ -1239,7 +1268,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
         <v>23</v>
       </c>
@@ -1250,7 +1279,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
         <v>24</v>
       </c>
@@ -1261,7 +1290,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
         <v>25</v>
       </c>
@@ -1272,7 +1301,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
         <v>26</v>
       </c>
@@ -1283,7 +1312,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
         <v>27</v>
       </c>
@@ -1294,7 +1323,7 @@
         <v>2.0000000000000001E-4</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
         <v>28</v>
       </c>
@@ -1305,7 +1334,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
         <v>29</v>
       </c>
@@ -1316,7 +1345,7 @@
         <v>7.000000000000001E-4</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
         <v>30</v>
       </c>
@@ -1396,7 +1425,7 @@
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="B39" s="12"/>
       <c r="C39" s="9">
@@ -1668,7 +1697,7 @@
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A64" s="1" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="B64" s="1" t="s">
         <v>2</v>
@@ -1679,7 +1708,7 @@
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A65" s="1" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="B65" s="1" t="s">
         <v>2</v>
@@ -1741,7 +1770,7 @@
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A71" s="1" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="B71" s="1" t="s">
         <v>2</v>

</xml_diff>